<commit_message>
docs(gtm): compare DA pricing with funding routes
</commit_message>
<xml_diff>
--- a/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
+++ b/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Schedule" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55Cr Cohort" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Scale" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding Comparison" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execution Schedule'!$A$8:$K$25</definedName>
@@ -111,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -160,6 +161,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3076,4 +3080,435 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day-one liquidity by funding route</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Illustrative pre-GST comparison. Debt release is a repayment of existing borrowing, not a transaction cost or economic profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Comparison input</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Pool principal (₹cr)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Existing debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>35.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Discounted DA price per ₹1</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>PTC MRR</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>PTC transaction cost</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>0.0125</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PTC cash enhancement</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse advance rate</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Warehouse setup cost on funding</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Other DA all-inclusive comparator</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Gross cash / funding (₹cr)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Upfront cost or support (₹cr)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Net before debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Residual cash after debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Continuing economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>DA Base at par</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>'55Cr Cohort'!H5/100</f>
+        <v/>
+      </c>
+      <c r="D16" s="17">
+        <f>B16-C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>D16-$B$5</f>
+        <v/>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Sold share has no funding liability; seller gives up future spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>DA Premium at par</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>'55Cr Cohort'!H6/100</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>B17-C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>D17-$B$5</f>
+        <v/>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Adds conditional registry and duty allowances</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>DA Premium + one RTO action</t>
+        </is>
+      </c>
+      <c r="B18" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
+        <f>'55Cr Cohort'!H7/100</f>
+        <v/>
+      </c>
+      <c r="D18" s="17">
+        <f>B18-C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="17">
+        <f>D18-$B$5</f>
+        <v/>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Adds one modelled ₹100 RTO action per vehicle</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>DA Base at ₹99</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>B4*B6</f>
+        <v/>
+      </c>
+      <c r="C19" s="15">
+        <f>('55Cr Cohort'!B13+MAX(5,MIN(B4*B6,25)*40/100+MAX(B4*B6-25,0)*30/100)+SUM('55Cr Cohort'!B19:B23))/100</f>
+        <v/>
+      </c>
+      <c r="D19" s="15">
+        <f>B19-C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="15">
+        <f>D19-$B$5</f>
+        <v/>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>One price point reduces gross proceeds by ₹55L; execution fee adjusts slightly</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Other DA at assumed all-in 1.5%</t>
+        </is>
+      </c>
+      <c r="B20" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
+        <f>B4*B12</f>
+        <v/>
+      </c>
+      <c r="D20" s="17">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>D20-$B$5</f>
+        <v/>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Comparable only if 1.5% includes every external and platform item</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PTC with 10% MRR</t>
+        </is>
+      </c>
+      <c r="B21" s="15">
+        <f>B4*(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C21" s="15">
+        <f>B4*B8</f>
+        <v/>
+      </c>
+      <c r="D21" s="15">
+        <f>B21-C21</f>
+        <v/>
+      </c>
+      <c r="E21" s="15">
+        <f>D21-$B$5</f>
+        <v/>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Retained exposure and waterfall economics continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>PTC plus 5% cash enhancement</t>
+        </is>
+      </c>
+      <c r="B22" s="17">
+        <f>B4*(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C22" s="17">
+        <f>B4*B8+B4*B9</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>B22-C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="17">
+        <f>D22-$B$5</f>
+        <v/>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Retained exposure and cash support remain at risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>80% warehouse / term refinance</t>
+        </is>
+      </c>
+      <c r="B23" s="15">
+        <f>B4*B10</f>
+        <v/>
+      </c>
+      <c r="C23" s="15">
+        <f>B4*B10*B11</f>
+        <v/>
+      </c>
+      <c r="D23" s="15">
+        <f>B23-C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="15">
+        <f>D23-$B$5</f>
+        <v/>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Debt remains; annual interest at 8–11% is additional</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Co-lending for new production</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Not comparable</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Ex-ante future-origination route; not a sale of this seasoned pool</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CAssureRail — decision model — 16 September 2026&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(gtm): model 125 crore DA comparison
</commit_message>
<xml_diff>
--- a/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
+++ b/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55Cr Cohort" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Scale" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding Comparison" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="125Cr Comparison" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execution Schedule'!$A$8:$K$25</definedName>
@@ -112,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -164,6 +165,7 @@
     <xf numFmtId="10" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1926,7 +1928,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>AssureRail fees (₹L)</t>
+          <t>Platform/adviser fees (₹L)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2175,16 +2177,15 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>1.5% all-inclusive comparator</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>Alternative 1.5% fee + Base external</t>
+        </is>
+      </c>
+      <c r="F10" s="11">
+        <f>B12*1.5</f>
+        <v/>
       </c>
       <c r="G10" s="11">
-        <f>B12*1.5</f>
+        <f>SUM(B19:B23)</f>
         <v/>
       </c>
       <c r="H10" s="11">
@@ -2216,6 +2217,39 @@
       </c>
       <c r="B11" s="10">
         <f>B4*B5</f>
+        <v/>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Alternative 1.5% fee + Premium external</t>
+        </is>
+      </c>
+      <c r="F11" s="10">
+        <f>B12*1.5</f>
+        <v/>
+      </c>
+      <c r="G11" s="10">
+        <f>SUM(B19:B25)</f>
+        <v/>
+      </c>
+      <c r="H11" s="10">
+        <f>F11+G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="14">
+        <f>H11/(B12*100)</f>
+        <v/>
+      </c>
+      <c r="J11" s="10">
+        <f>H11/B4</f>
+        <v/>
+      </c>
+      <c r="K11" s="15">
+        <f>B12-H11/100</f>
+        <v/>
+      </c>
+      <c r="L11" s="15">
+        <f>K11-B8</f>
         <v/>
       </c>
     </row>
@@ -2554,17 +2588,17 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>1.5% comparator (₹L)</t>
+          <t>Alternative 1.5% fee (₹L)</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Base variance to comparator (₹L)</t>
+          <t>Alternative Base total (₹L)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Premium variance to comparator (₹L)</t>
+          <t>Base saving vs alternative (₹L)</t>
         </is>
       </c>
     </row>
@@ -2605,11 +2639,11 @@
         <v/>
       </c>
       <c r="J10" s="11">
-        <f>E10-I10</f>
+        <f>I10+$B$5</f>
         <v/>
       </c>
       <c r="K10" s="11">
-        <f>G10-I10</f>
+        <f>J10-E10</f>
         <v/>
       </c>
     </row>
@@ -2650,11 +2684,11 @@
         <v/>
       </c>
       <c r="J11" s="10">
-        <f>E11-I11</f>
+        <f>I11+$B$5</f>
         <v/>
       </c>
       <c r="K11" s="10">
-        <f>G11-I11</f>
+        <f>J11-E11</f>
         <v/>
       </c>
     </row>
@@ -2695,11 +2729,11 @@
         <v/>
       </c>
       <c r="J12" s="11">
-        <f>E12-I12</f>
+        <f>I12+$B$5</f>
         <v/>
       </c>
       <c r="K12" s="11">
-        <f>G12-I12</f>
+        <f>J12-E12</f>
         <v/>
       </c>
     </row>
@@ -2740,11 +2774,11 @@
         <v/>
       </c>
       <c r="J13" s="10">
-        <f>E13-I13</f>
+        <f>I13+$B$5</f>
         <v/>
       </c>
       <c r="K13" s="10">
-        <f>G13-I13</f>
+        <f>J13-E13</f>
         <v/>
       </c>
     </row>
@@ -2785,11 +2819,11 @@
         <v/>
       </c>
       <c r="J14" s="11">
-        <f>E14-I14</f>
+        <f>I14+$B$5</f>
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>G14-I14</f>
+        <f>J14-E14</f>
         <v/>
       </c>
     </row>
@@ -2830,11 +2864,11 @@
         <v/>
       </c>
       <c r="J15" s="10">
-        <f>E15-I15</f>
+        <f>I15+$B$5</f>
         <v/>
       </c>
       <c r="K15" s="10">
-        <f>G15-I15</f>
+        <f>J15-E15</f>
         <v/>
       </c>
     </row>
@@ -2875,11 +2909,11 @@
         <v/>
       </c>
       <c r="J16" s="11">
-        <f>E16-I16</f>
+        <f>I16+$B$5</f>
         <v/>
       </c>
       <c r="K16" s="11">
-        <f>G16-I16</f>
+        <f>J16-E16</f>
         <v/>
       </c>
     </row>
@@ -2920,11 +2954,11 @@
         <v/>
       </c>
       <c r="J17" s="10">
-        <f>E17-I17</f>
+        <f>I17+$B$5</f>
         <v/>
       </c>
       <c r="K17" s="10">
-        <f>G17-I17</f>
+        <f>J17-E17</f>
         <v/>
       </c>
     </row>
@@ -2965,11 +2999,11 @@
         <v/>
       </c>
       <c r="J18" s="11">
-        <f>E18-I18</f>
+        <f>I18+$B$5</f>
         <v/>
       </c>
       <c r="K18" s="11">
-        <f>G18-I18</f>
+        <f>J18-E18</f>
         <v/>
       </c>
     </row>
@@ -3010,11 +3044,11 @@
         <v/>
       </c>
       <c r="J19" s="10">
-        <f>E19-I19</f>
+        <f>I19+$B$5</f>
         <v/>
       </c>
       <c r="K19" s="10">
-        <f>G19-I19</f>
+        <f>J19-E19</f>
         <v/>
       </c>
     </row>
@@ -3055,11 +3089,11 @@
         <v/>
       </c>
       <c r="J20" s="11">
-        <f>E20-I20</f>
+        <f>I20+$B$5</f>
         <v/>
       </c>
       <c r="K20" s="11">
-        <f>G20-I20</f>
+        <f>J20-E20</f>
         <v/>
       </c>
     </row>
@@ -3088,7 +3122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3208,7 +3242,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Other DA all-inclusive comparator</t>
+          <t>Alternative adviser/platform fee</t>
         </is>
       </c>
       <c r="B12" s="16" t="n">
@@ -3362,7 +3396,7 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Other DA at assumed all-in 1.5%</t>
+          <t>Other DA: 1.5% fee + Base external</t>
         </is>
       </c>
       <c r="B20" s="17">
@@ -3370,7 +3404,7 @@
         <v/>
       </c>
       <c r="C20" s="17">
-        <f>B4*B12</f>
+        <f>B4*B12+SUM('55Cr Cohort'!B19:B23)/100</f>
         <v/>
       </c>
       <c r="D20" s="17">
@@ -3383,22 +3417,22 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Comparable only if 1.5% includes every external and platform item</t>
+          <t>External and statutory costs added on the same Base scope</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>PTC with 10% MRR</t>
+          <t>Other DA: 1.5% fee + Premium external</t>
         </is>
       </c>
       <c r="B21" s="15">
-        <f>B4*(1-B7)</f>
+        <f>B4</f>
         <v/>
       </c>
       <c r="C21" s="15">
-        <f>B4*B8</f>
+        <f>B4*B12+SUM('55Cr Cohort'!B19:B25)/100</f>
         <v/>
       </c>
       <c r="D21" s="15">
@@ -3411,14 +3445,14 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Retained exposure and waterfall economics continue</t>
+          <t>Premium-scope external costs added separately</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>PTC plus 5% cash enhancement</t>
+          <t>PTC with 10% MRR</t>
         </is>
       </c>
       <c r="B22" s="17">
@@ -3426,7 +3460,7 @@
         <v/>
       </c>
       <c r="C22" s="17">
-        <f>B4*B8+B4*B9</f>
+        <f>B4*B8</f>
         <v/>
       </c>
       <c r="D22" s="17">
@@ -3439,22 +3473,22 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Retained exposure and cash support remain at risk</t>
+          <t>Retained exposure and waterfall economics continue</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>80% warehouse / term refinance</t>
+          <t>PTC plus 5% cash enhancement</t>
         </is>
       </c>
       <c r="B23" s="15">
-        <f>B4*B10</f>
+        <f>B4*(1-B7)</f>
         <v/>
       </c>
       <c r="C23" s="15">
-        <f>B4*B10*B11</f>
+        <f>B4*B8+B4*B9</f>
         <v/>
       </c>
       <c r="D23" s="15">
@@ -3467,32 +3501,834 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Debt remains; annual interest at 8–11% is additional</t>
+          <t>Retained exposure and cash support remain at risk</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
+          <t>80% warehouse / term refinance</t>
+        </is>
+      </c>
+      <c r="B24" s="17">
+        <f>B4*B10</f>
+        <v/>
+      </c>
+      <c r="C24" s="17">
+        <f>B4*B10*B11</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>B24-C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="17">
+        <f>D24-$B$5</f>
+        <v/>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Debt remains; annual interest at 8–11% is additional</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>Co-lending for new production</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Not comparable</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Ex-ante future-origination route; not a sale of this seasoned pool</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CAssureRail — decision model — 16 September 2026&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="64" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>₹125 crore EV cohort comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Primary case scales the ₹55 crore EV population to about 9,375 loans. All transaction-cost values are pre-GST planning assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Case input</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Gross cash/funding (₹cr)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Cost/support (₹cr)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Net before debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Residual cash after debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Continuing economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Pool principal (₹cr)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>125</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>DA Base at par</t>
+        </is>
+      </c>
+      <c r="F4" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="G4" s="17">
+        <f>(B19+B32)/100</f>
+        <v/>
+      </c>
+      <c r="H4" s="17">
+        <f>F4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="17">
+        <f>H4-$B$16</f>
+        <v/>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Sold share has no funding liability; future spread surrendered</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Sellers</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>DA Premium at par</t>
+        </is>
+      </c>
+      <c r="F5" s="15">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
+        <f>(B19+B33)/100</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
+        <f>F5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="15">
+        <f>H5-$B$16</f>
+        <v/>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Adds registry and duty allowances</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Average outstanding per loan (₹L)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>1.3333333333</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>DA Premium + one RTO action</t>
+        </is>
+      </c>
+      <c r="F6" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="G6" s="17">
+        <f>(B19+B34)/100</f>
+        <v/>
+      </c>
+      <c r="H6" s="17">
+        <f>F6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="17">
+        <f>H6-$B$16</f>
+        <v/>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Adds one modelled RTO action per vehicle</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Existing debt release</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>DA Base at ₹99</t>
+        </is>
+      </c>
+      <c r="F7" s="15">
+        <f>B4*0.99</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>(B17+MAX(5,MIN(F7,25)*40/100+MAX(F7-25,0)*30/100)+B32)/100</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
+        <f>F7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="15">
+        <f>H7-$B$16</f>
+        <v/>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>One price point reduces gross proceeds by ₹1.25cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Fixed-stage rate per admitted loan (₹)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Other DA: 1.5% fee + Base external</t>
+        </is>
+      </c>
+      <c r="F8" s="17">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="G8" s="17">
+        <f>B4*B11+B32/100</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>F8-G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="17">
+        <f>H8-$B$16</f>
+        <v/>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Like-for-like Base external costs added to fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Fixed-stage minimum per seller (₹L)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Other DA: 1.5% fee + Premium external</t>
+        </is>
+      </c>
+      <c r="F9" s="15">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>B4*B11+B33/100</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
+        <f>F9-G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="15">
+        <f>H9-$B$16</f>
+        <v/>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Like-for-like Premium external costs added to fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Escrow/bank/VAN working base (₹L)</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>PTC with 10% MRR</t>
+        </is>
+      </c>
+      <c r="F10" s="17">
+        <f>B4*0.90</f>
+        <v/>
+      </c>
+      <c r="G10" s="17">
+        <f>B4*0.0125</f>
+        <v/>
+      </c>
+      <c r="H10" s="17">
+        <f>F10-G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="17">
+        <f>H10-$B$16</f>
+        <v/>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Retained exposure and waterfall economics continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Alternative adviser/platform fee</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>PTC plus 5% cash enhancement</t>
+        </is>
+      </c>
+      <c r="F11" s="15">
+        <f>B4*0.90</f>
+        <v/>
+      </c>
+      <c r="G11" s="15">
+        <f>B4*0.0125+B4*0.05</f>
+        <v/>
+      </c>
+      <c r="H11" s="15">
+        <f>F11-G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="15">
+        <f>H11-$B$16</f>
+        <v/>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Retained exposure and cash support remain at risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>80% warehouse / term refinance</t>
+        </is>
+      </c>
+      <c r="F12" s="17">
+        <f>B4*0.80</f>
+        <v/>
+      </c>
+      <c r="G12" s="17">
+        <f>B4*0.80*0.01</f>
+        <v/>
+      </c>
+      <c r="H12" s="17">
+        <f>F12-G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="17">
+        <f>H12-$B$16</f>
+        <v/>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>₹100cr debt remains; annual interest at 8–11% is ₹8–11cr at full utilisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Derived case values</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Co-lending for new production</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>Not comparable</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Not a sale of this seasoned pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Admitted loans</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>B4*100/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Loans per seller</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>B14/B5</f>
+        <v/>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Loan-count sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Existing debt release (₹cr)</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>B4*B7</f>
+        <v/>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Admitted loans</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Fixed stages (₹L)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Base external (₹L)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>AssureRail + Base total (₹L)</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Share of ₹125cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Fixed-stage fees (₹L)</t>
+        </is>
+      </c>
+      <c r="B17" s="10">
+        <f>B5*MAX(B9,B15*B8/100000)</f>
+        <v/>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>4125</v>
+      </c>
+      <c r="F17" s="10">
+        <f>$B$5*MAX($B$9,E17/$B$5*$B$8/100000)</f>
+        <v/>
+      </c>
+      <c r="G17" s="10">
+        <f>E17*40/100000+$B$10+10.5+0.53+E17*25/100000</f>
+        <v/>
+      </c>
+      <c r="H17" s="10">
+        <f>F17+$B$18+G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="14">
+        <f>H17/($B$4*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Candidate execution fee (₹L)</t>
+        </is>
+      </c>
+      <c r="B18" s="11">
+        <f>MAX(5,MIN(B4,25)*40/100+MAX(B4-25,0)*30/100)</f>
+        <v/>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>9375</v>
+      </c>
+      <c r="F18" s="11">
+        <f>$B$5*MAX($B$9,E18/$B$5*$B$8/100000)</f>
+        <v/>
+      </c>
+      <c r="G18" s="11">
+        <f>E18*40/100000+$B$10+10.5+0.53+E18*25/100000</f>
+        <v/>
+      </c>
+      <c r="H18" s="11">
+        <f>F18+$B$18+G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="16">
+        <f>H18/($B$4*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Total AssureRail fees (₹L)</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>B17+B18</f>
+        <v/>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F19" s="10">
+        <f>$B$5*MAX($B$9,E19/$B$5*$B$8/100000)</f>
+        <v/>
+      </c>
+      <c r="G19" s="10">
+        <f>E19*40/100000+$B$10+10.5+0.53+E19*25/100000</f>
+        <v/>
+      </c>
+      <c r="H19" s="10">
+        <f>F19+$B$18+G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="14">
+        <f>H19/($B$4*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>External-cost build</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>External item</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Working amount (₹L)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Derivation</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Fresh bureau pulls</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>B14*40/100000</f>
+        <v/>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Loan count × ₹40</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Escrow, bank and VAN</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Negotiated cohort working base</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Transaction counsel and seller schedules</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Common scope plus five schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>ROC filing and support</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Five sellers</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>NeSL submissions</t>
+        </is>
+      </c>
+      <c r="B27" s="10">
+        <f>B14*25/100000</f>
+        <v/>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Loan count × ₹25 if fresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Conditional registry actions</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Conditional assignment duty</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>One RTO action per vehicle</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>B14*100/100000</f>
+        <v/>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Premium if required</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Base external total</t>
+        </is>
+      </c>
+      <c r="B32" s="21">
+        <f>SUM(B23:B27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Premium external total</t>
+        </is>
+      </c>
+      <c r="B33" s="21">
+        <f>SUM(B23:B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Premium + RTO external total</t>
+        </is>
+      </c>
+      <c r="B34" s="21">
+        <f>SUM(B23:B30)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gtm): add 300 crore CFO treasury pitch
</commit_message>
<xml_diff>
--- a/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
+++ b/docs/gtm/AssureRail_DA_40_30_Bps_Scenario_Model_2026-09-16.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Scale" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding Comparison" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="125Cr Comparison" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="300Cr CFO Pitch" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execution Schedule'!$A$8:$K$25</definedName>
@@ -792,7 +793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -918,6 +919,18 @@
       <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Model before implementation. Existing rate-card versions, accepted quotes and contracts remain unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CFO sales case</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>The 300Cr CFO Pitch sheet models seasoning contribution, Full-service proceeds, price sensitivity, future spread surrendered and a 1.5% fee-only alternative.</t>
         </is>
       </c>
     </row>
@@ -4347,4 +4360,784 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>₹300 crore CFO and treasury case</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Illustrative 36-month, 24% reducing-balance EV pool with 70% of tenor remaining. Replace every yellow input with the NBFC’s actual data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Treasury input</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Full-service cost build</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Total NBFC loan book (₹cr)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Service/cost item</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Working amount (₹L)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Current pool selected for sale (₹cr)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Fresh bureau pulls</t>
+        </is>
+      </c>
+      <c r="F5" s="10">
+        <f>B19*40/100000</f>
+        <v/>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>3,000 × ₹40 planning rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Indicative PSL share</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Escrow, bank and VAN</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Negotiated large-programme base</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Average current outstanding per loan (₹L)</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Transaction counsel and four closing rounds</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Accepted capped scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Original tenor (months)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>ROC filing and support</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>One seller</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elapsed months</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>NeSL submissions</t>
+        </is>
+      </c>
+      <c r="F9" s="10">
+        <f>B19*25/100000</f>
+        <v/>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>If fresh submission required</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Borrower yield, reducing balance</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Conditional registry work</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Full scope allowance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Cost of funds</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Conditional assignment duty</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Counsel-confirmed treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Upfront acquisition/origination cost</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Risk-based travel and field checks</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Accepted sample design</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Annual servicing/operations cost</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Additional buyer counsel</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Only if contractually seller-borne</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Existing debt release as share of pool</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Monitoring activation plus 12 months</t>
+        </is>
+      </c>
+      <c r="F14" s="11">
+        <f>0.75+(0.25+B19*5/100000)*12</f>
+        <v/>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>One reporting unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Alternative adviser/platform fee</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Optional one RTO action per vehicle</t>
+        </is>
+      </c>
+      <c r="F15" s="10">
+        <f>B19*100/100000</f>
+        <v/>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Excluded unless required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Realised credit loss/write-off to date (₹cr)</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Full external cost, excluding RTO</t>
+        </is>
+      </c>
+      <c r="F17" s="21">
+        <f>SUM(F5:F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Seasoning economics</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Optional RTO addition</t>
+        </is>
+      </c>
+      <c r="F18" s="21">
+        <f>F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Admitted loans</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>B5*100/B7</f>
+        <v/>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Fixed-stage fees</t>
+        </is>
+      </c>
+      <c r="F19" s="21">
+        <f>B19*500/100000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Remaining months</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
+        <f>B8-B9</f>
+        <v/>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Execution fee at par</t>
+        </is>
+      </c>
+      <c r="F20" s="21">
+        <f>MAX(5,MIN(B5,25)*40/100+MAX(B5-25,0)*30/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Monthly borrower rate</t>
+        </is>
+      </c>
+      <c r="B21" s="10">
+        <f>B10/12</f>
+        <v/>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Total AssureRail fees at par</t>
+        </is>
+      </c>
+      <c r="F21" s="21">
+        <f>F19+F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Original EMI factor</t>
+        </is>
+      </c>
+      <c r="B22" s="11">
+        <f>B21*(1+B21)^B8/((1+B21)^B8-1)</f>
+        <v/>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Full-service total at par, excluding RTO</t>
+        </is>
+      </c>
+      <c r="F22" s="21">
+        <f>F17+F21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Outstanding/original-principal ratio after elapsed months</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>(1+B21)^B9-B22*((1+B21)^B9-1)/B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Reconstructed original principal (₹cr)</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>B5/B23</f>
+        <v/>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Purchase price per ₹100</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Gross consideration (₹cr)</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Full-service cost (₹L)</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Net sale cash (₹cr)</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Net cash as % of ₹300cr</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Cash after modelled debt release (₹cr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Monthly scheduled collections (₹cr)</t>
+        </is>
+      </c>
+      <c r="B25" s="10">
+        <f>B24*B22</f>
+        <v/>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="F25" s="10">
+        <f>$B$5*E25/100</f>
+        <v/>
+      </c>
+      <c r="G25" s="10">
+        <f>$F$19+MAX(5,MIN(F25,25)*40/100+MAX(F25-25,0)*30/100)+$F$17</f>
+        <v/>
+      </c>
+      <c r="H25" s="10">
+        <f>F25-G25/100</f>
+        <v/>
+      </c>
+      <c r="I25" s="14">
+        <f>H25/$B$5</f>
+        <v/>
+      </c>
+      <c r="J25" s="10">
+        <f>H25-$B$5*$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Gross interest earned to date (₹cr)</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>B25*B9-(B24-B5)</f>
+        <v/>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>99</v>
+      </c>
+      <c r="F26" s="11">
+        <f>$B$5*E26/100</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
+        <f>$F$19+MAX(5,MIN(F26,25)*40/100+MAX(F26-25,0)*30/100)+$F$17</f>
+        <v/>
+      </c>
+      <c r="H26" s="11">
+        <f>F26-G26/100</f>
+        <v/>
+      </c>
+      <c r="I26" s="16">
+        <f>H26/$B$5</f>
+        <v/>
+      </c>
+      <c r="J26" s="11">
+        <f>H26-$B$5*$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Sum of monthly opening balances to date (₹cr-month)</t>
+        </is>
+      </c>
+      <c r="B27" s="10">
+        <f>B24*(((1+B21)^B9-1)/B21-B22/B21*(((1+B21)^B9-1)/B21-B9))</f>
+        <v/>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="F27" s="10">
+        <f>$B$5*E27/100</f>
+        <v/>
+      </c>
+      <c r="G27" s="10">
+        <f>$F$19+MAX(5,MIN(F27,25)*40/100+MAX(F27-25,0)*30/100)+$F$17</f>
+        <v/>
+      </c>
+      <c r="H27" s="10">
+        <f>F27-G27/100</f>
+        <v/>
+      </c>
+      <c r="I27" s="14">
+        <f>H27/$B$5</f>
+        <v/>
+      </c>
+      <c r="J27" s="10">
+        <f>H27-$B$5*$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Funding cost to date (₹cr)</t>
+        </is>
+      </c>
+      <c r="B28" s="11">
+        <f>B27*B11/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Acquisition/origination cost (₹cr)</t>
+        </is>
+      </c>
+      <c r="B29" s="10">
+        <f>B24*B12</f>
+        <v/>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Alternative 1.5% fee at par (₹L)</t>
+        </is>
+      </c>
+      <c r="F29" s="21">
+        <f>B5*1.5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Servicing/operations cost to date (₹cr)</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>B27*B13/12</f>
+        <v/>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Alternative plus same Full external costs (₹L)</t>
+        </is>
+      </c>
+      <c r="F30" s="21">
+        <f>F29+F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Illustrative contribution earned (₹cr)</t>
+        </is>
+      </c>
+      <c r="B31" s="10">
+        <f>B26-B28-B29-B30-B16</f>
+        <v/>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Alternative net cash at par (₹cr)</t>
+        </is>
+      </c>
+      <c r="F31" s="21">
+        <f>B5-F30/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Contribution as % of current ₹300cr balance</t>
+        </is>
+      </c>
+      <c r="B32" s="16">
+        <f>B31/B5</f>
+        <v/>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>AssureRail net-cash advantage (₹cr)</t>
+        </is>
+      </c>
+      <c r="F32" s="21">
+        <f>H25-F31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Contribution as % of reconstructed original principal</t>
+        </is>
+      </c>
+      <c r="B33" s="14">
+        <f>B31/B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Remaining contractual gross interest (₹cr)</t>
+        </is>
+      </c>
+      <c r="B34" s="11">
+        <f>B25*B20-B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Sum of future monthly opening balances (₹cr-month)</t>
+        </is>
+      </c>
+      <c r="B35" s="10">
+        <f>B5*(((1+B21)^B20-1)/B21)-B25/B21*(((1+B21)^B20-1)/B21-B20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Future funding cost (₹cr)</t>
+        </is>
+      </c>
+      <c r="B36" s="11">
+        <f>B35*B11/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Future servicing/operations cost (₹cr)</t>
+        </is>
+      </c>
+      <c r="B37" s="10">
+        <f>B35*B13/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Future contribution retained if held, before losses/tax (₹cr)</t>
+        </is>
+      </c>
+      <c r="B38" s="11">
+        <f>B34-B36-B37</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CAssureRail — decision model — 16 September 2026&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>